<commit_message>
Align app with the first-interview hearing sheet
- DB migration v2: contact, shift pattern, required benefits, holiday preference, priorities,
  current job status, other offers, disclosure scope, considerations
- Hearing answers feed matching (benefit checks, 5-day week, wage target vs floor, priority weights)
- Condition-sheet Excel template rebuilt in the hearing sheet's order; AI extraction reads checkboxes
- Today's tasks show other-offer deadlines; new 'ヒアリング' tab on seeker page

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SoLj5wH7BCM62ZskcRbuaW
</commit_message>
<xml_diff>
--- a/shushoku-matching/frontend/public/joken-template.xlsx
+++ b/shushoku-matching/frontend/public/joken-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="111">
   <si>
     <t>項目</t>
   </si>
@@ -43,43 +43,91 @@
     <t>例：1990/4/1</t>
   </si>
   <si>
+    <t>都道府県</t>
+  </si>
+  <si>
+    <t>例：大阪府</t>
+  </si>
+  <si>
+    <t>市区町村</t>
+  </si>
+  <si>
+    <t>お住まいの地域。例：堺市</t>
+  </si>
+  <si>
+    <t>最寄り駅</t>
+  </si>
+  <si>
     <t>電話番号</t>
   </si>
   <si>
     <t>メールアドレス</t>
   </si>
   <si>
-    <t>住所</t>
-  </si>
-  <si>
-    <t>通勤・勤務地</t>
-  </si>
-  <si>
-    <t>都道府県</t>
-  </si>
-  <si>
-    <t>例：大阪府</t>
-  </si>
-  <si>
-    <t>市区町村</t>
-  </si>
-  <si>
-    <t>例：堺市</t>
-  </si>
-  <si>
-    <t>最寄り駅</t>
+    <t>連絡方法</t>
+  </si>
+  <si>
+    <t>電話/メール</t>
+  </si>
+  <si>
+    <t>連絡のとりやすい時間帯</t>
+  </si>
+  <si>
+    <t>例：平日18時以降</t>
+  </si>
+  <si>
+    <t>紹介元・担当者</t>
+  </si>
+  <si>
+    <t>記入日</t>
+  </si>
+  <si>
+    <t>例：2026/10/14</t>
+  </si>
+  <si>
+    <t>就業条件</t>
+  </si>
+  <si>
+    <t>希望職種</t>
+  </si>
+  <si>
+    <t>介護職員・ヘルパー/看護師/准看護師/生活相談員/ケアマネジャー/機能訓練指導員/その他</t>
+  </si>
+  <si>
+    <t>希望雇用形態</t>
+  </si>
+  <si>
+    <t>正社員/契約社員/パート・アルバイト/派遣</t>
+  </si>
+  <si>
+    <t>希望施設</t>
+  </si>
+  <si>
+    <t>特養/老健/デイ/有料/GH/訪問/病院/その他（問わない場合は空欄）</t>
+  </si>
+  <si>
+    <t>週の勤務日数上限</t>
+  </si>
+  <si>
+    <t>例：5</t>
+  </si>
+  <si>
+    <t>希望勤務時間帯</t>
+  </si>
+  <si>
+    <t>日勤のみ/早番・遅番可/夜勤可/オンコール可</t>
   </si>
   <si>
     <t>通勤可能な市区町村</t>
   </si>
   <si>
-    <t>例：和泉市,高石市（カンマ区切り）</t>
+    <t>例：和泉市,高石市</t>
   </si>
   <si>
     <t>通勤手段</t>
   </si>
   <si>
-    <t>例：車,公共交通</t>
+    <t>自転車/徒歩/公共交通/車</t>
   </si>
   <si>
     <t>通勤時間の上限（分）</t>
@@ -88,157 +136,208 @@
     <t>例：40</t>
   </si>
   <si>
-    <t>希望の仕事</t>
-  </si>
-  <si>
-    <t>希望職種</t>
-  </si>
-  <si>
-    <t>例：介護</t>
-  </si>
-  <si>
-    <t>希望職務</t>
-  </si>
-  <si>
-    <t>介護職/生活相談員/看護職/ケアマネ/機能訓練/送迎/調理/事務/その他</t>
-  </si>
-  <si>
-    <t>希望施設</t>
-  </si>
-  <si>
-    <t>特養/老健/介護医療院/GH/有料/サ高住/デイ/訪問/小多機/障害/病院/保育/その他</t>
-  </si>
-  <si>
-    <t>希望しない施設</t>
-  </si>
-  <si>
-    <t>希望雇用形態</t>
-  </si>
-  <si>
-    <t>例：正社員,パート</t>
+    <t>勤務に制約のある曜日・時間帯</t>
+  </si>
+  <si>
+    <t>理由の記入は不要</t>
+  </si>
+  <si>
+    <t>避けたい条件・譲れない条件</t>
+  </si>
+  <si>
+    <t>例：夜勤は月4回まで</t>
+  </si>
+  <si>
+    <t>夜勤回数の上限（月）</t>
+  </si>
+  <si>
+    <t>例：4（0=不可）</t>
+  </si>
+  <si>
+    <t>志望動機・転職理由</t>
+  </si>
+  <si>
+    <t>給与・待遇条件</t>
   </si>
   <si>
     <t>賃金形態</t>
   </si>
   <si>
-    <t>月給/時給/日給/年俸</t>
+    <t>月給/時給</t>
+  </si>
+  <si>
+    <t>希望給与</t>
+  </si>
+  <si>
+    <t>例：25万</t>
   </si>
   <si>
     <t>希望賃金</t>
   </si>
   <si>
-    <t>例：22万</t>
-  </si>
-  <si>
-    <t>働き方</t>
-  </si>
-  <si>
-    <t>勤務可能時間（開始）</t>
-  </si>
-  <si>
-    <t>例：8:30</t>
-  </si>
-  <si>
-    <t>勤務可能時間（終了）</t>
-  </si>
-  <si>
-    <t>例：18:00</t>
-  </si>
-  <si>
-    <t>夜勤・交替制</t>
+    <t>最低希望ライン。例：22万</t>
+  </si>
+  <si>
+    <t>現在（直近）の給与</t>
+  </si>
+  <si>
+    <t>任意・参考</t>
+  </si>
+  <si>
+    <t>必須の手当・待遇</t>
+  </si>
+  <si>
+    <t>交通費支給/資格手当/夜勤手当/住宅手当/賞与あり/退職金制度</t>
+  </si>
+  <si>
+    <t>休日・休暇の希望</t>
+  </si>
+  <si>
+    <t>週休2日以上 など</t>
+  </si>
+  <si>
+    <t>固定休日希望（曜日）</t>
+  </si>
+  <si>
+    <t>例：日曜</t>
+  </si>
+  <si>
+    <t>希望年間休日</t>
+  </si>
+  <si>
+    <t>例：105</t>
+  </si>
+  <si>
+    <t>優先順位</t>
+  </si>
+  <si>
+    <t>重視する順に。例：給与,勤務地,休日</t>
+  </si>
+  <si>
+    <t>資格・経験</t>
+  </si>
+  <si>
+    <t>保有資格</t>
+  </si>
+  <si>
+    <t>看護師/准看護師/介護福祉士/実務者研修/初任者研修/ケアマネジャー/社会福祉士/喀痰吸引等研修 など</t>
+  </si>
+  <si>
+    <t>運転免許</t>
+  </si>
+  <si>
+    <t>普通（AT限定なし）/普通（AT限定）/なし</t>
+  </si>
+  <si>
+    <t>経験年数</t>
+  </si>
+  <si>
+    <t>例：3</t>
+  </si>
+  <si>
+    <t>経験した現場</t>
+  </si>
+  <si>
+    <t>施設系/在宅系/病院/クリニック/未経験</t>
+  </si>
+  <si>
+    <t>夜勤経験</t>
+  </si>
+  <si>
+    <t>例：あり（月4回・3年）</t>
+  </si>
+  <si>
+    <t>看護師の診療科・病棟経験</t>
+  </si>
+  <si>
+    <t>看護師の場合</t>
+  </si>
+  <si>
+    <t>外国籍</t>
+  </si>
+  <si>
+    <t>はい/いいえ</t>
+  </si>
+  <si>
+    <t>在留資格</t>
+  </si>
+  <si>
+    <t>特定技能1号/技能実習/永住者 など</t>
+  </si>
+  <si>
+    <t>在留期限</t>
+  </si>
+  <si>
+    <t>日本語能力</t>
+  </si>
+  <si>
+    <t>N1〜N5/なし</t>
+  </si>
+  <si>
+    <t>JFT-Basic合格</t>
+  </si>
+  <si>
+    <t>介護日本語評価試験</t>
+  </si>
+  <si>
+    <t>合格/未受験</t>
+  </si>
+  <si>
+    <t>入職希望時期・現職状況</t>
+  </si>
+  <si>
+    <t>現職の状況</t>
+  </si>
+  <si>
+    <t>在職中/離職中</t>
+  </si>
+  <si>
+    <t>退職予定日</t>
+  </si>
+  <si>
+    <t>就業可能日</t>
+  </si>
+  <si>
+    <t>入職希望時期</t>
+  </si>
+  <si>
+    <t>転職活動の状況</t>
+  </si>
+  <si>
+    <t>応募前/他社に応募中（○社）/面接中/内定あり</t>
+  </si>
+  <si>
+    <t>他社内定の回答期限</t>
+  </si>
+  <si>
+    <t>他の紹介会社の利用</t>
+  </si>
+  <si>
+    <t>あり/なし</t>
+  </si>
+  <si>
+    <t>面接・職場見学が可能な曜日・時間帯</t>
+  </si>
+  <si>
+    <t>現在の勤務先への在籍確認</t>
   </si>
   <si>
     <t>可/不可</t>
   </si>
   <si>
-    <t>夜勤回数の上限（月）</t>
-  </si>
-  <si>
-    <t>例：4（0=不可）</t>
-  </si>
-  <si>
-    <t>夜勤専従希望</t>
-  </si>
-  <si>
-    <t>はい/いいえ</t>
-  </si>
-  <si>
-    <t>週の勤務日数上限</t>
-  </si>
-  <si>
-    <t>例：5</t>
-  </si>
-  <si>
-    <t>希望年間休日</t>
-  </si>
-  <si>
-    <t>例：105</t>
-  </si>
-  <si>
-    <t>就業可能日</t>
-  </si>
-  <si>
-    <t>例：2026/11/1</t>
-  </si>
-  <si>
-    <t>資格・経験</t>
-  </si>
-  <si>
-    <t>保有資格</t>
-  </si>
-  <si>
-    <t>例：介護福祉士,普通自動車免許</t>
-  </si>
-  <si>
-    <t>経験年数</t>
-  </si>
-  <si>
-    <t>例：3</t>
-  </si>
-  <si>
-    <t>職務経歴</t>
-  </si>
-  <si>
-    <t>優先順位</t>
-  </si>
-  <si>
-    <t>例：家から近いこと、夜勤なし</t>
-  </si>
-  <si>
-    <t>外国籍の方</t>
-  </si>
-  <si>
-    <t>外国籍</t>
-  </si>
-  <si>
-    <t>在留資格</t>
-  </si>
-  <si>
-    <t>例：特定技能1号</t>
-  </si>
-  <si>
-    <t>在留期限</t>
-  </si>
-  <si>
-    <t>日本語能力</t>
-  </si>
-  <si>
-    <t>N1〜N5/なし</t>
-  </si>
-  <si>
-    <t>介護日本語評価試験</t>
-  </si>
-  <si>
-    <t>合格/未</t>
-  </si>
-  <si>
-    <t>技能試験</t>
-  </si>
-  <si>
-    <t>例：介護技能評価試験</t>
+    <t>紹介先へ提供してよい情報の範囲</t>
+  </si>
+  <si>
+    <t>氏名を伏せた概要のみ/氏名を含めて提供可</t>
   </si>
   <si>
     <t>その他</t>
+  </si>
+  <si>
+    <t>配慮してほしいこと</t>
+  </si>
+  <si>
+    <t>任意。健康・障害等は本人が希望する場合のみ</t>
   </si>
   <si>
     <t>備考</t>
@@ -645,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -716,23 +815,23 @@
         <v>4</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>4</v>
@@ -741,328 +840,328 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="2" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="4" t="s">
+    </row>
+    <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="B15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>4</v>
+      <c r="B16" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>4</v>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>46</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>47</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>4</v>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>4</v>
@@ -1073,90 +1172,277 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>4</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>4</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>77</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>84</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>85</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>87</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>88</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>93</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>94</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>98</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>102</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>104</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>107</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>109</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>